<commit_message>
Implemented Excel Data Driven Testing
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/LoginData.xlsx
+++ b/src/test/resources/testdata/LoginData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TLTUser\OneDrive\Desktop\SeleniumTraining\demoapp\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{094CD772-BF72-45FA-BAE4-D59800D46556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15EBDA49-5044-408B-8177-1835A61F70DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3300" yWindow="3396" windowWidth="17280" windowHeight="8964" xr2:uid="{2D58542D-E341-45EB-B46E-5AA960131D33}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{2D58542D-E341-45EB-B46E-5AA960131D33}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
   <si>
     <t>Username</t>
   </si>
@@ -54,6 +54,9 @@
   </si>
   <si>
     <t>Wrong123</t>
+  </si>
+  <si>
+    <t>wronguser@test.com</t>
   </si>
 </sst>
 </file>
@@ -452,7 +455,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07619F28-A07C-43B2-8FD2-33C856D9E046}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
@@ -479,10 +482,19 @@
         <v>4</v>
       </c>
     </row>
+    <row r="4" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="mailto:jabdul@thoughtlinetech.com" xr:uid="{CD4348E0-0F41-4BE4-B39F-13197E0C5D9E}"/>
-    <hyperlink ref="A3" r:id="rId2" display="mailto:jabdul@thoughtlinetech.com" xr:uid="{15047533-DD0B-4B6E-80AA-7F9A072156B5}"/>
+    <hyperlink ref="A2" r:id="rId1" display="mailto:jabdul@thoughtlinetech.com" xr:uid="{BF07A533-0AF8-420D-BDD9-C6B978E390FA}"/>
+    <hyperlink ref="A3" r:id="rId2" display="mailto:jabdul@thoughtlinetech.com" xr:uid="{86F449E3-8A7A-4AFF-AA3D-7455817E27C9}"/>
+    <hyperlink ref="A4" r:id="rId3" display="mailto:wronguser@test.com" xr:uid="{AAE1FA49-721B-4E45-BCFA-1E058DFBF570}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Implemented Excel driven login validation with PASS and FAIL scenarios
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/LoginData.xlsx
+++ b/src/test/resources/testdata/LoginData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TLTUser\OneDrive\Desktop\SeleniumTraining\demoapp\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15EBDA49-5044-408B-8177-1835A61F70DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32DAFA53-6234-481C-866B-E3408B2E4E07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{2D58542D-E341-45EB-B46E-5AA960131D33}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
   <si>
     <t>Username</t>
   </si>
@@ -57,6 +57,15 @@
   </si>
   <si>
     <t>wronguser@test.com</t>
+  </si>
+  <si>
+    <t>Expected</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>FAIL</t>
   </si>
 </sst>
 </file>
@@ -72,17 +81,17 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <u/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
+      <b/>
       <sz val="11"/>
-      <color theme="10"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -107,18 +116,18 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -455,46 +464,58 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07619F28-A07C-43B2-8FD2-33C856D9E046}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="C2" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="3" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="C3" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="4" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>3</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="mailto:jabdul@thoughtlinetech.com" xr:uid="{BF07A533-0AF8-420D-BDD9-C6B978E390FA}"/>
-    <hyperlink ref="A3" r:id="rId2" display="mailto:jabdul@thoughtlinetech.com" xr:uid="{86F449E3-8A7A-4AFF-AA3D-7455817E27C9}"/>
-    <hyperlink ref="A4" r:id="rId3" display="mailto:wronguser@test.com" xr:uid="{AAE1FA49-721B-4E45-BCFA-1E058DFBF570}"/>
+    <hyperlink ref="A2" r:id="rId1" display="mailto:jabdul@thoughtlinetech.com" xr:uid="{A3342BCE-D7B7-4C22-B6C8-0A060B84CBDA}"/>
+    <hyperlink ref="A3" r:id="rId2" display="mailto:jabdul@thoughtlinetech.com" xr:uid="{53006D75-4E7E-46A6-A83F-3B4C015457E8}"/>
+    <hyperlink ref="A4" r:id="rId3" display="mailto:wronguser@test.com" xr:uid="{90F41095-3374-4BF9-B8ED-C5D147CFF805}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>